<commit_message>
test case 7 modified
</commit_message>
<xml_diff>
--- a/lms/src/test/resources/data.xlsx
+++ b/lms/src/test/resources/data.xlsx
@@ -4,12 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="2"/>
+    <workbookView windowWidth="10668" windowHeight="9000" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
   <si>
     <t>user email</t>
   </si>
@@ -53,6 +55,66 @@
   </si>
   <si>
     <t>da@gmail.com</t>
+  </si>
+  <si>
+    <t>page</t>
+  </si>
+  <si>
+    <t>limit</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>ispinned</t>
+  </si>
+  <si>
+    <t>sortBy</t>
+  </si>
+  <si>
+    <t>sortOrder</t>
+  </si>
+  <si>
+    <t>API</t>
+  </si>
+  <si>
+    <t>qa</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>asc</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
+  <si>
+    <t>desc</t>
+  </si>
+  <si>
+    <t>Selenium</t>
+  </si>
+  <si>
+    <t>updatedAt</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>isPinned</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>QA</t>
   </si>
 </sst>
 </file>
@@ -1310,4 +1372,271 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="6"/>
+  <cols>
+    <col min="6" max="6" width="16.4444444444444" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>